<commit_message>
References workbook: single A2 explanation on all three sheets, matching Peter's edit to sheet 1
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_references.xlsx
+++ b/textbook_examples/mod01_references.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Relative" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Absolute" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Several crops" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Relative referencing example" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Absolute referencing example" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Absolute referencing example 2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E11"/>
+  <dimension ref="A1:E9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -512,7 +512,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>The formula in column D multiplies the two cells beside it. Copy it down and BOTH references move with it — row 5 uses row 5, row 6 uses row 6.</t>
+          <t>In this worksheet we have five loads of grain.  Each load has a different size in bushels (col B) and price per bushel (col C).  We want to calculate the value of each load by multiplying bushels times price.  To do so, we can just write B5*C5 in cell D5 and the copy that equation into cells D6-D9.</t>
         </is>
       </c>
     </row>
@@ -650,18 +650,11 @@
       </c>
     </row>
     <row r="10" ht="18" customHeight="1"/>
-    <row r="11" ht="32" customHeight="1">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>Read column E downwards: B5*C5, then B6*C6, then B7*C7. Both references step down one row at a time — each load uses its own bushels and its own price. This is what a reference does if you leave it alone.</t>
-        </is>
-      </c>
-    </row>
+    <row r="11" ht="18" customHeight="1"/>
     <row r="12" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="1">
     <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A11:E11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -673,7 +666,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D13"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -692,7 +685,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Here the conversion factor lives in ONE cell (B4). Every formula has to point at that same cell, so we lock it with dollar signs: $B$4.</t>
+          <t>Now we want the same five loads in tonnes rather than bushels.  The conversion factor sits in one cell (B4), and every load needs that same cell.  If we write B7*B4 and copy it down, the B4 part drifts to B5, B6 and the answers go wrong.  Writing B7*$B$4 instead locks the factor in place while the bushels still move.</t>
         </is>
       </c>
     </row>
@@ -826,17 +819,10 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1"/>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>Read column D downwards: the B7 part steps down to B8, B9 … but $B$4 never changes. Without the dollar signs it would drift to B5, B6, B7 and the answers would be wrong. Type B4 and press F4 (Windows) or ⌘T (Mac) to add the dollar signs.</t>
-        </is>
-      </c>
-    </row>
+    <row r="13" ht="18" customHeight="1"/>
     <row r="14" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A13:D13"/>
+  <mergeCells count="1">
     <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -849,7 +835,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F13"/>
+  <dimension ref="A1:F11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -870,7 +856,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Each crop has its own factor, side by side in row 4. One formula fills all three columns: lock the ROW so it always looks up to row 4, but leave the column free so each column finds its own crop.</t>
+          <t>Now each crop has its own conversion factor, sitting side by side in row 4.  We want one formula that fills all three columns.  Writing $B7*C$4 locks the column on the bushels (so every crop reads column B) and locks the row on the factors (so every load reads row 4) — but leaves the other half of each free to move.</t>
         </is>
       </c>
     </row>
@@ -1056,17 +1042,10 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1"/>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>The one formula is =$B7*C$4, filled across and down. $B keeps every column looking left to the bushels. C$4 keeps every row looking up to row 4 — and because the column letter is free, wheat reads C4, barley D4, oats E4.</t>
-        </is>
-      </c>
-    </row>
+    <row r="13" ht="18" customHeight="1"/>
     <row r="14" ht="18" customHeight="1"/>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="A13:F13"/>
+  <mergeCells count="1">
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Rename references workbook tabs to Ex1/Ex2/Ex3
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_references.xlsx
+++ b/textbook_examples/mod01_references.xlsx
@@ -7,9 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Relative referencing example" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Absolute referencing example" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Absolute referencing example 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Ex1 (relative)" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Ex2 (absolute)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Ex3 (absolute)" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>

</xml_diff>

<commit_message>
Ex3 of the references workbook: two crops with factors beneath their own columns
Adopts Peter's revision into the generator and updates the A2 explanation to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0165WQeoaB3CPsnpvD7o3Yah
</commit_message>
<xml_diff>
--- a/textbook_examples/mod01_references.xlsx
+++ b/textbook_examples/mod01_references.xlsx
@@ -835,15 +835,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
     <col width="13" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
@@ -856,28 +856,12 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Now each crop has its own conversion factor, sitting side by side in row 4.  We want one formula that fills all three columns.  Writing $B7*C$4 locks the column on the bushels (so every crop reads column B) and locks the row on the factors (so every load reads row 4) — but leaves the other half of each free to move.</t>
+          <t>Now we have two crops, and each has its own conversion factor.  The factors sit in row 14, directly underneath the column they belong to.  Writing B7*B$14 locks the row (so every load reads row 14) but leaves the column free — so the wheat column reads B14 and the barley column reads C14.</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1"/>
-    <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="10" t="inlineStr">
-        <is>
-          <t>Tonnes per bushel →</t>
-        </is>
-      </c>
-      <c r="B4" s="5" t="inlineStr"/>
-      <c r="C4" s="11" t="n">
-        <v>0.027216</v>
-      </c>
-      <c r="D4" s="11" t="n">
-        <v>0.021772</v>
-      </c>
-      <c r="E4" s="11" t="n">
-        <v>0.017237</v>
-      </c>
-    </row>
+    <row r="4" ht="18" customHeight="1"/>
     <row r="5" ht="18" customHeight="1"/>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="3" t="inlineStr">
@@ -887,27 +871,27 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Bushels</t>
+          <t>Wheat_bu</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>wheat_tons</t>
+          <t>Barley_bu</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>barley_tons</t>
+          <t>Wheat_tons</t>
         </is>
       </c>
       <c r="E6" s="4" t="inlineStr">
         <is>
-          <t>oats_tons</t>
+          <t>Barley_tons</t>
         </is>
       </c>
       <c r="F6" s="4" t="inlineStr">
         <is>
-          <t>The formula in C</t>
+          <t>The formula in D</t>
         </is>
       </c>
     </row>
@@ -920,20 +904,19 @@
       <c r="B7" s="6" t="n">
         <v>500</v>
       </c>
-      <c r="C7" s="13">
-        <f>$B7*C$4</f>
-        <v/>
+      <c r="C7" s="6" t="n">
+        <v>200</v>
       </c>
       <c r="D7" s="13">
-        <f>$B7*D$4</f>
+        <f>B7*B$14</f>
         <v/>
       </c>
       <c r="E7" s="13">
-        <f>$B7*E$4</f>
+        <f>C7*C$14</f>
         <v/>
       </c>
       <c r="F7" s="9">
-        <f>_xlfn.FORMULATEXT(C7)</f>
+        <f>_xlfn.FORMULATEXT(D7)</f>
         <v/>
       </c>
     </row>
@@ -946,20 +929,19 @@
       <c r="B8" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="C8" s="13">
-        <f>$B8*C$4</f>
-        <v/>
+      <c r="C8" s="6" t="n">
+        <v>300</v>
       </c>
       <c r="D8" s="13">
-        <f>$B8*D$4</f>
+        <f>B8*B$14</f>
         <v/>
       </c>
       <c r="E8" s="13">
-        <f>$B8*E$4</f>
+        <f>C8*C$14</f>
         <v/>
       </c>
       <c r="F8" s="9">
-        <f>_xlfn.FORMULATEXT(C8)</f>
+        <f>_xlfn.FORMULATEXT(D8)</f>
         <v/>
       </c>
     </row>
@@ -972,20 +954,19 @@
       <c r="B9" s="6" t="n">
         <v>2500</v>
       </c>
-      <c r="C9" s="13">
-        <f>$B9*C$4</f>
-        <v/>
+      <c r="C9" s="6" t="n">
+        <v>600</v>
       </c>
       <c r="D9" s="13">
-        <f>$B9*D$4</f>
+        <f>B9*B$14</f>
         <v/>
       </c>
       <c r="E9" s="13">
-        <f>$B9*E$4</f>
+        <f>C9*C$14</f>
         <v/>
       </c>
       <c r="F9" s="9">
-        <f>_xlfn.FORMULATEXT(C9)</f>
+        <f>_xlfn.FORMULATEXT(D9)</f>
         <v/>
       </c>
     </row>
@@ -998,20 +979,19 @@
       <c r="B10" s="6" t="n">
         <v>5000</v>
       </c>
-      <c r="C10" s="13">
-        <f>$B10*C$4</f>
-        <v/>
+      <c r="C10" s="6" t="n">
+        <v>800</v>
       </c>
       <c r="D10" s="13">
-        <f>$B10*D$4</f>
+        <f>B10*B$14</f>
         <v/>
       </c>
       <c r="E10" s="13">
-        <f>$B10*E$4</f>
+        <f>C10*C$14</f>
         <v/>
       </c>
       <c r="F10" s="9">
-        <f>_xlfn.FORMULATEXT(C10)</f>
+        <f>_xlfn.FORMULATEXT(D10)</f>
         <v/>
       </c>
     </row>
@@ -1024,26 +1004,38 @@
       <c r="B11" s="6" t="n">
         <v>8000</v>
       </c>
-      <c r="C11" s="13">
-        <f>$B11*C$4</f>
-        <v/>
+      <c r="C11" s="6" t="n">
+        <v>1500</v>
       </c>
       <c r="D11" s="13">
-        <f>$B11*D$4</f>
+        <f>B11*B$14</f>
         <v/>
       </c>
       <c r="E11" s="13">
-        <f>$B11*E$4</f>
+        <f>C11*C$14</f>
         <v/>
       </c>
       <c r="F11" s="9">
-        <f>_xlfn.FORMULATEXT(C11)</f>
+        <f>_xlfn.FORMULATEXT(D11)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1"/>
     <row r="13" ht="18" customHeight="1"/>
-    <row r="14" ht="18" customHeight="1"/>
+    <row r="14" ht="18" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
+        <is>
+          <t>Tons/bu</t>
+        </is>
+      </c>
+      <c r="B14" s="11" t="n">
+        <v>0.027216</v>
+      </c>
+      <c r="C14" s="11" t="n">
+        <v>0.021772</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A2:F2"/>

</xml_diff>